<commit_message>
Drop the 2 family trusts from scope per instruction
Reword the badge, Exec Summary data-confidence legend, Group Summary
label, and Notes sheet so the 16-entity model reads as the full
intended scope rather than "2 entities still pending" — the trusts
are excluded by decision, not a gap to fill later.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C4h9XrSFz9TM2sZz9NNf79
</commit_message>
<xml_diff>
--- a/output/Sandhu_Group_Interactive_Dashboard.xlsx
+++ b/output/Sandhu_Group_Interactive_Dashboard.xlsx
@@ -1182,7 +1182,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>DRAFT MANAGEMENT REPORT — 16/18 ENTITIES REBUILT FROM SOURCE  ·  3-YEAR P&amp;L, ALL VALIDATED TO THE PENNY</t>
+          <t>DRAFT MANAGEMENT REPORT — ALL 16 ENTITIES IN SCOPE REBUILT FROM SOURCE  ·  3-YEAR P&amp;L, ALL VALIDATED TO THE PENNY</t>
         </is>
       </c>
       <c r="C2" s="3" t="n"/>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>P&amp;L, 16/18 entities — every entity rebuilt fresh from its raw CaseWare WTB (FY2023–FY2025) and independently cross-validated: FY2025 Net Income matches the project's Validation Log exactly for all 16, to the penny.</t>
+          <t>P&amp;L, all 16 entities in scope (2 family trusts excluded per instruction) — every entity rebuilt fresh from its raw CaseWare WTB (FY2023–FY2025) and independently cross-validated: FY2025 Net Income matches the project's Validation Log exactly, to the penny.</t>
         </is>
       </c>
       <c r="M18" s="1" t="n"/>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>Both family trusts (~$4–$10/yr activity per the handoff) and one unexpected entity found in the Taxprep data (9475-3381 Québec Inc., no WTB supplied) — not yet modeled.</t>
+          <t>One unexpected entity found in the Taxprep data (9475-3381 Québec Inc.) has no WTB supplied and is not modeled — needs confirmation on whether it belongs in the group.</t>
         </is>
       </c>
       <c r="M22" s="1" t="n"/>
@@ -5586,7 +5586,7 @@
       <c r="A5" s="1" t="n"/>
       <c r="B5" s="46" t="inlineStr">
         <is>
-          <t>16-entity group total (per Entity Register) — 2 family trusts pending WTB files</t>
+          <t>16-entity group total (per Entity Register) — full scope (2 family trusts excluded)</t>
         </is>
       </c>
       <c r="C5" s="1" t="n"/>
@@ -6127,7 +6127,7 @@
     <row r="3">
       <c r="A3" s="50" t="inlineStr">
         <is>
-          <t>Scope: 16 of 18 entities. Every one of these was rebuilt fresh from its raw CaseWare WTB export in this session (not carried over from any prior file) and covers 3 fiscal years: FY2023, FY2024, FY2025.</t>
+          <t>Scope: all 16 entities (both family trusts — Gurpreet Sandhu Trust, Harpreet Sandhu Trust — excluded from scope per instruction; ~$4-$10/yr activity per the handoff, immaterial). Every one of these was rebuilt fresh from its raw CaseWare WTB export in this session (not carried over from any prior file) and covers 3 fiscal years: FY2023, FY2024, FY2025.</t>
         </is>
       </c>
       <c r="B3" s="1" t="n"/>
@@ -6139,7 +6139,7 @@
     <row r="5">
       <c r="A5" s="50" t="inlineStr">
         <is>
-          <t>Missing: both family trusts (Gurpreet Sandhu Trust, Harpreet Sandhu Trust — ~$4-$10/yr activity per the handoff, no files supplied) and Sandhu &amp; Sandhu Enr.'s Corporate Taxprep export (its WTB was supplied and is included).</t>
+          <t>Missing: Sandhu &amp; Sandhu Enr.'s Corporate Taxprep export (its WTB was supplied and is included).</t>
         </is>
       </c>
       <c r="B5" s="1" t="n"/>

</xml_diff>